<commit_message>
Update documentation and scripts for improved CI and dataset handling
- Revise README.md to reflect updated CI job statuses and test coverage.
- Enhance ASSUMPTIONS.md with details on model artifacts and dataset management via Git LFS.
- Modify checklist_data.py to include results from a 60-epoch A100 run.
- Update download_datasets.py to handle tqdm import gracefully, ensuring compatibility across environments.
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-23 12:18:16 India Standard Time</t>
+          <t>2026-09-23 17:54:43 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>torch.autocast + GradScaler on CUDA; bf16 on CPU (no scaler needed, since bf16 has float32 exponent range so gradients cannot underflow). Active in the full 30-epoch A100 run (73.98% top-1 / 90.18% top-5).</t>
+          <t>torch.autocast + GradScaler on CUDA; bf16 on CPU (no scaler needed, since bf16 has float32 exponent range so gradients cannot underflow). Active in the full 60-epoch A100 run: 77.66% top-1 / 91.52% top-5, validated 8/8 by validate.py.</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>clip_grad_norm_ after unscaling (order matters with AMP). Grad norm logged per epoch. Active in the full 30-epoch A100 run.</t>
+          <t>clip_grad_norm_ after unscaling (order matters with AMP). Grad norm logged per epoch; 8 of 60 epochs hit non-finite grads, absorbed by GradScaler as designed.</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Cosine with linear warmup (default), plus onecycle/step/plateau. Per-batch vs per-epoch stepping handled explicitly. Active in the full 30-epoch A100 run.</t>
+          <t>Cosine with linear warmup (default), plus onecycle/step/plateau. Per-batch vs per-epoch stepping handled explicitly. Cosine + 5% warmup over the full 60-epoch run.</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1207,12 @@
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>models/optimization/export_tensorrt.py</t>
+          <t>models/optimization/export_tensorrt.py; benchmarks/reports/BENCHMARKS_GPU.md</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Export + benchmark implemented and GPU-gated. NOT EXECUTED: no NVIDIA GPU on the build machine. Documented in docs/ASSUMPTIONS.md.</t>
+          <t>EXECUTED on an A100 (TensorRT 11.3). fp16: 0.729 ms p50, 1369 img/s, 46.0 MB. fp32: 1.059 ms, 972 img/s. Handles the TRT 8/10/11 API differences by probing attributes. INT8 via TRT not built - refused rather than faked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update deliverables checklist and add unit tests for worker lifecycle and tasks
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-24 11:16:14 India Standard Time</t>
+          <t>2026-09-25 20:10:59 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>EXECUTED on an A100 (TensorRT 11.3). fp16: 0.729 ms p50, 1369 img/s, 46.0 MB. fp32: 1.059 ms, 972 img/s. Handles the TRT 8/10/11 API differences by probing attributes. INT8 via TRT not built - refused rather than faked.</t>
+          <t>EXECUTED on an A100 (TensorRT 11.3.0.99). All three precisions built and verified: int8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms, 1066 img/s, 46.0 MB; fp32 1.298 ms, 822 img/s, 91.5 MB. Handles the TRT 8/10/11 API differences by probing attributes. INT8 needed a separate QDQ graph: fp32 biases, symmetric, percentile calibration, stem conv excluded.</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 3 models, p50/p95/p99 with environment recorded. Key finding: dynamic INT8 is 13x SLOWER than fp32 on this CPU; static QDQ is 1.4x slower and 3.9x smaller.</t>
+          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 3 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 is 13x SLOWER than fp32 on this CPU, static QDQ is 1.4x slower and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>83% overall; critical paths 85-100%. Routers 97-100%, validators 92%, image_processing 98%, schemas/responses 97-98%.</t>
+          <t>95.7% on api/ and 100% on worker/, the two halves of the request path; 88.8% across api+worker+models. The async batch endpoint was the last gap at 82.6% and is now fully covered, including the URL fetch with its SSRF checks, the soft-timeout partial-results path and the completion callback at both the helper and its call site.</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Lint, type-check, test, coverage gate, Docker build and security scan.</t>
+          <t>Eight jobs: lint, tests on 3.11 and 3.12, security scan, image build, end-to-end against the deployed stack, real model export. Plus release.yml (publishes attested, scanned images on a version tag) and drift-watch.yml (weekly retraining decision, verified by a manual run).</t>
         </is>
       </c>
     </row>
@@ -3308,12 +3308,12 @@
       </c>
       <c r="F76" s="13" t="inlineStr">
         <is>
-          <t>docker/Dockerfile.api, docker/Dockerfile.worker</t>
+          <t>Dockerfile, docker/Dockerfile.worker, docker/Dockerfile.gpu</t>
         </is>
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>Builder stage keeps compilers out of the runtime image.</t>
+          <t>Builder stage keeps compilers out of the runtime image. A third Dockerfile builds the CUDA/TensorRT serving image.</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G113" s="13" t="inlineStr">
         <is>
-          <t>83.5% overall; critical paths 85-100% (routers 97-100%, validators 92%, image_processing 98%). The gap is GPU-only and lifespan code.</t>
+          <t>Zero modules below 85% on the critical path, counting worker/ as well as api/: 95.7% on api/, 100% on worker/tasks.py and worker/celery_app.py. 88.8% across the whole repo. The weakest critical-path module is health.py at 86.8%. What remains under 85% is training and MLOps code no request touches: registry.py (a CLI, not imported by api/ or worker/), train_classifier.py, retraining.py, dataset.py, tracking.py.</t>
         </is>
       </c>
     </row>
@@ -4648,12 +4648,12 @@
       </c>
       <c r="F116" s="13" t="inlineStr">
         <is>
-          <t>docs/TECHNICAL.md, docker-compose.prod.yml</t>
+          <t>k8s/, docs/TECHNICAL.md, docker-compose.prod.yml</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>Stateless API, Redis-backed distributed rate limiting, independent worker scaling. The per-process similarity index is documented as the one component that does not yet scale out.</t>
+          <t>Stateless API, Redis-backed distributed rate limiting, independent worker scaling, and a pgvector-backed similarity index shared by every replica (the per-process default does not scale, which is why the Kubernetes config sets SIMILARITY_BACKEND=pgvector). Verified on a kind cluster: the HPA scaled ml-api from 1 pod to 2 under a forced target.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update deliverables checklist with improved test coverage details and documentation references
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25 20:10:59 India Standard Time</t>
+          <t>2026-09-25 21:17:01 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>95.7% on api/ and 100% on worker/, the two halves of the request path; 88.8% across api+worker+models. The async batch endpoint was the last gap at 82.6% and is now fully covered, including the URL fetch with its SSRF checks, the soft-timeout partial-results path and the completion callback at both the helper and its call site.</t>
+          <t>95.9% across api/ and worker/ together, the request path end to end: 95.7% on api/, 100% on worker/. 89.3% repo-wide including the training and MLOps code. The async batch endpoint was the last gap at 82.6% and is now fully covered, including the URL fetch with its SSRF checks, the soft-timeout partial-results path and the completion callback at both the helper and its call site.</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="F64" s="13" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_routes.py, tests/integration/</t>
+          <t>tests/unit/test_api_routes.py, tests/integration/, scripts/smoke_test_api.py</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Plus a verified live run through the Docker stack.</t>
+          <t>Plus a verified live run through the Docker stack: 30 checks over every documented endpoint, 30/30 through the gateway and 30/30 against the API's own port. It is a script rather than a transcript, so it reruns against any deployment and exits non-zero on a failure.</t>
         </is>
       </c>
     </row>
@@ -3969,12 +3969,12 @@
       </c>
       <c r="F95" s="13" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md</t>
+          <t>docs/DEPLOYMENT.md, k8s/README.md</t>
         </is>
       </c>
       <c r="G95" s="13" t="inlineStr">
         <is>
-          <t>First run, production checklist, scaling guide with measured sizing, monitoring, model rollout/rollback, troubleshooting, backup and recovery.</t>
+          <t>First run, production checklist, scaling guide with measured sizing, a Kubernetes section covering when to move, prerequisites, what changes from Compose and how to verify it, then monitoring, model rollout/rollback, troubleshooting, backup and recovery. The manifests have their own README with the cluster evidence.</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>Architecture diagram, middleware ordering rationale, layering.</t>
+          <t>A diagram per deployment target, Compose and Kubernetes, with the middleware ordering rationale and layering. TECHNICAL.md §6 covers why the cluster topology differs: HPA instead of a typed replica count, ingress instead of the gateway container, fetched rather than baked-in artifacts, and migrations in an init container.</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G113" s="13" t="inlineStr">
         <is>
-          <t>Zero modules below 85% on the critical path, counting worker/ as well as api/: 95.7% on api/, 100% on worker/tasks.py and worker/celery_app.py. 88.8% across the whole repo. The weakest critical-path module is health.py at 86.8%. What remains under 85% is training and MLOps code no request touches: registry.py (a CLI, not imported by api/ or worker/), train_classifier.py, retraining.py, dataset.py, tracking.py.</t>
+          <t>Zero modules below 85% on the critical path, counting worker/ as well as api/: 95.9% across the two, 95.7% on api/, 100% on worker/tasks.py and worker/celery_app.py. 89.3% across the whole repo. The weakest critical-path module is health.py at 86.8%. What remains under 85% is training and MLOps code no request touches: registry.py (a CLI, not imported by api/ or worker/), train_classifier.py, retraining.py, dataset.py, tracking.py.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor model benchmarks and validation reports
- Updated ONNX export reports to include new models: resnet50-tiny-imagenet and resnet50.
- Adjusted validation report timestamps and metrics for resnet50 and resnet50-tiny-imagenet.
- Enhanced accuracy and latency metrics in validation reports, including new checks for inference errors and calibration.
- Revised API documentation to reflect updated inference timings for models.
- Modified assumptions and technical documentation to align with new performance metrics and quantization results.
- Updated model cards for resnet50, resnet50-embed, resnet50-tiny-imagenet, and yolov8n with revised latency and accuracy figures.
- Added new quantization accuracy report for resnet50-tiny-imagenet.
- Corrected checklist data to reflect changes in performance monitoring and benchmarking results.
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25 21:17:01 India Standard Time</t>
+          <t>2026-09-25 22:06:19 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 3 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 is 13x SLOWER than fp32 on this CPU, static QDQ is 1.4x slower and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
+          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 4 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 will not even load on this CPU (no ConvInteger kernel), static QDQ is 1.07x to 2.30x slower depending on the model and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>13 Prometheus metrics (counters, histograms, gauges) covering requests, inference, cache, model loads and batch jobs. 11 alert rules validated by promtool, each alerting on a user-visible symptom rather than a cause and carrying a description of what to do about it. 22-panel Grafana dashboard, auto-provisioned. All VERIFIED live against the running stack.</t>
+          <t>15 Prometheus metrics (counters, histograms, gauges) covering requests, inference, cache, model loads and batch jobs. 11 alert rules validated by promtool, each alerting on a user-visible symptom rather than a cause and carrying a description of what to do about it. 22-panel Grafana dashboard, auto-provisioned. All VERIFIED live against the running stack.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>p99 at batch 1: resnet50 131ms, yolov8n 235ms, embed 388ms. All inside the 1s budget; the slowest is ~4x inside it.</t>
+          <t>p99 at batch 1: resnet50 146ms, resnet50-tiny-imagenet 93ms, yolov8n 166ms, embed 63ms. Every model and both precisions stay inside the 1s budget; the slowest overall is yolov8n INT8 at 338ms, 3x inside it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor documentation and code comments for clarity and consistency
- Updated README.md in k8s directory to correct spelling of "artefacts" and improve phrasing for better readability.
- Revised model cards for ResNet-50, including changes to terminology (e.g., "artefact" instead of "artifact") and improved explanations of model performance and quantization.
- Enhanced clarity in YOLOv8n detection model card by refining descriptions and correcting terminology.
- Improved comments in quantization script to clarify the implications of dynamic quantization and provide better guidance on model loading issues.
- Adjusted sample README to maintain consistent language regarding file handling.
- Updated checklist_data.py to provide clearer insights on benchmark findings related to INT8 quantization.
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25 22:06:19 India Standard Time</t>
+          <t>2026-09-25 22:22:21 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 4 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 will not even load on this CPU (no ConvInteger kernel), static QDQ is 1.07x to 2.30x slower depending on the model and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
+          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 4 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 will not load as configured (uint8 activations against int8 weights is not a registered ConvInteger kernel; QUInt8 weights fix it), static QDQ is 1.07x to 2.30x slower depending on the model and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update deliverables checklist and improve API documentation with new authentication endpoint details
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25 22:22:21 India Standard Time</t>
+          <t>2026-09-25 22:55:06 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>OpenAPI 3.1, 18 paths / 37 schemas. Importable directly into Postman.</t>
+          <t>OpenAPI 3.1, 19 paths / 40 schemas. Importable directly into Postman.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update performance metrics in documentation and checklist
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-25 22:55:06 India Standard Time</t>
+          <t>2026-09-26 14:35:36 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -927,12 +927,12 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>scripts/prepare_models.py; models/artifacts/yolov8n.onnx</t>
+          <t>scripts/prepare_models.py; models/validation/coco_eval.py; benchmarks/reports/coco_eval.json</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>YOLOv8n trained on COCO. Verified on a real photo: detected 4 people + 1 bus with correct boxes in original image coordinates.</t>
+          <t>YOLOv8n with Ultralytics COCO weights. Measured on 500 COCO val2017 images through the serving path: 0.392 mAP50-95, 0.536 mAP50 (pycocotools).</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>models/training/train_classifier.py</t>
+          <t>models/training/train_classifier.py; benchmarks/reports/resnet50_training_history.json</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>torch.autocast + GradScaler on CUDA; bf16 on CPU (no scaler needed, since bf16 has float32 exponent range so gradients cannot underflow). Active in the full 60-epoch A100 run: 77.66% top-1 / 91.52% top-5, validated 8/8 by validate.py.</t>
+          <t>torch.autocast fp16 with GradScaler on CUDA (bf16 on CPU). 60 epochs on an A100: 78.91% top-1, 92.12% top-5, identical when the exported ONNX model is scored through the serving path on all 10,000 validation images.</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>clip_grad_norm_ after unscaling (order matters with AMP). Grad norm logged per epoch; 8 of 60 epochs hit non-finite grads, absorbed by GradScaler as designed.</t>
+          <t>clip_grad_norm_ at 1.0 after unscaling (the order matters with AMP). Grad norm and loss scale logged per epoch; the end-of-epoch loss scale drops at epochs 12, 18, 25, 43 and 49, where GradScaler skipped non-finite steps.</t>
         </is>
       </c>
     </row>
@@ -1067,12 +1067,12 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>data/tiny-imagenet-200; models/training/dataset.py</t>
+          <t>scripts/download_datasets.py; models/training/dataset.py</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>200 classes / 120k images downloaded. Custom val loader reads val_annotations.txt, because ImageFolder silently mislabels that split (the provided starter script has this bug).</t>
+          <t>All 200 classes, 100,000 training and 10,000 validation images (120,203 files, 240 MB). The validation loader reads val_annotations.txt because ImageFolder labels that split as one class, a bug in the provided starter script.</t>
         </is>
       </c>
     </row>
@@ -1137,12 +1137,12 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>models/optimization/quantize.py; benchmarks/reports/quantization.json</t>
+          <t>models/optimization/quantize.py; benchmarks/reports/quantization.json; benchmarks/reports/int8_fidelity.json</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>All 3 models quantized. resnet50 97.4-&gt;24.5 MB (3.97x), yolov8n 12.2-&gt;3.3 MB (3.67x), resnet50-embed 89.6-&gt;22.6 MB (3.97x).</t>
+          <t>All 4 models, static QDQ, uint8 with percentile calibration (chosen by measurement, benchmarks/reports/int8_recipes.json): resnet50 3.92x smaller, resnet50-tiny-imagenet 3.91x, resnet50-embed 3.91x, yolov8n 3.67x (convolutions only, COCO-calibrated; 0.388 against 0.392 mAP50-95). The fine-tuned classifier loses 0.53 points of top-1 on 10,000 images. INT8 is selectable per request and the default for none; tests/integration/test_quantized_fidelity.py checks every INT8 model against fp32 in CI.</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1172,12 @@
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>models/optimization/export_onnx.py</t>
+          <t>models/optimization/export_onnx.py; scripts/verify_onnx_parity.py; benchmarks/reports/onnx_export.json</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>All 3 exported and numerically verified against PyTorch (max abs diff &lt; 4e-6). Uses the legacy exporter: torch 2.9's dynamo path ignored dynamic_axes (breaking batching) and split weights into a sidecar file.</t>
+          <t>All 4 exported and checked against PyTorch on real images; parity recorded for each in onnx_export.json. Uses the legacy exporter: torch 2.9's dynamo path ignored dynamic_axes and split weights into a sidecar file.</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1207,12 @@
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>models/optimization/export_tensorrt.py; benchmarks/reports/BENCHMARKS_GPU.md</t>
+          <t>models/optimization/export_tensorrt.py; benchmarks/reports/tensorrt.json</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>EXECUTED on an A100 (TensorRT 11.3.0.99). All three precisions built and verified: int8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms, 1066 img/s, 46.0 MB; fp32 1.298 ms, 822 img/s, 91.5 MB. Handles the TRT 8/10/11 API differences by probing attributes. INT8 needed a separate QDQ graph: fp32 biases, symmetric, percentile calibration, stem conv excluded.</t>
+          <t>Built and verified on an A100 (TensorRT 11.3.0.99) for the fine-tuned classifier: INT8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms; fp32 1.298 ms. The other three models have CPU INT8 only; building their engines needs another GPU session.</t>
         </is>
       </c>
     </row>
@@ -1242,12 +1242,12 @@
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>benchmarks/reports/BENCHMARKS.md</t>
+          <t>models/optimization/benchmark.py; benchmarks/reports/BENCHMARKS.md</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>fp32 ONNX vs INT8 static, batch 1 and 4, all 4 models, p50/p95/p99 with environment recorded, plus fp32/fp16/int8 TensorRT engines on an A100. Key findings: dynamic INT8 will not load as configured (uint8 activations against int8 weights is not a registered ConvInteger kernel; QUInt8 weights fix it), static QDQ is 1.07x to 2.30x slower depending on the model and 3.9x smaller, and on GPU int8 matches fp16 on latency while halving engine size.</t>
+          <t>fp32 and INT8 ONNX for all 4 models at batch 1 and 4, 100 runs per case interleaved across models, plus TensorRT fp32/fp16/INT8. INT8 (uint8, percentile calibration) on this CPU: 1.7x to 2.5x faster than fp32 for the three ResNets, 1.33x slower for yolov8n, 3.67x to 3.92x smaller.</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>models/validation/validate.py</t>
+          <t>models/validation/validate.py; benchmarks/reports/validation.json</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>8 checks: artifacts, determinism, batch invariance, output sanity, robustness, accuracy, calibration (ECE), latency. Caught 2 real bugs during development.</t>
+          <t>Artifacts, determinism, batch invariance, output sanity, robustness, inference errors, accuracy, calibration and latency. All 4 models pass; the fine-tuned model scores 78.91% top-1 on 10,000 images.</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>models/validation/ab_test.py</t>
+          <t>models/validation/ab_test.py; benchmarks/reports/ab_test.json</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Paired McNemar test, confidence interval on the accuracy delta, deterministic hash-based traffic splitting, and required-sample-size guidance.</t>
+          <t>Paired McNemar test with a confidence interval, latency comparison, hash-based traffic splitting. name:version@runtime compares runtimes of one model. Run on all 10,000 validation images, fp32 against INT8: 78.91% against 78.38%, p = 0.002, keep fp32.</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>models/validation/drift.py</t>
+          <t>models/validation/drift.py; benchmarks/reports/drift_report.json; benchmarks/reports/drift_report_shift.json</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>KS test, chi-square and PSI. Requires BOTH significance and a meaningful effect size, so a large sample cannot produce alert spam. Verified on a 200k-sample case.</t>
+          <t>KS test, chi-square and PSI, requiring significance and an effect size. Run on real images: a Tiny-ImageNet control shows no drift in any of 12 tests; against COCO photos, 8 of 12 tests drift, severity high, confidence 0.668 to 0.373 (PSI 1.51).</t>
         </is>
       </c>
     </row>
@@ -1382,12 +1382,12 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>models/validation/regression.py</t>
+          <t>models/validation/regression.py; benchmarks/baselines.json; benchmarks/reports/regression.json</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Baseline store with per-metric tolerances (absolute for accuracy, relative for latency) and hardware fingerprinting. Verified it catches an injected 150% regression.</t>
+          <t>Baselines with per-metric tolerances and hardware fingerprinting. Baselines for all 4 models at 100 iterations. Accuracy gates pass; latency gates are documented as needing dedicated hardware, because this laptop varies 30% within minutes (evidence in docs/TECHNICAL.md section 7).</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Verified 200, 5 objects detected.</t>
+          <t>Verified live through the gateway, in both the dev and production stacks.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>Verified: 3 models with defaults per task.</t>
+          <t>Lists every registered model with its default per task.</t>
         </is>
       </c>
     </row>
@@ -2509,12 +2509,12 @@
       </c>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>monitoring/prometheus/alerts.yml; monitoring/grafana/</t>
+          <t>api/middleware/monitoring.py; monitoring/</t>
         </is>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>15 Prometheus metrics (counters, histograms, gauges) covering requests, inference, cache, model loads and batch jobs. 11 alert rules validated by promtool, each alerting on a user-visible symptom rather than a cause and carrying a description of what to do about it. 22-panel Grafana dashboard, auto-provisioned. All VERIFIED live against the running stack.</t>
+          <t>Prometheus metrics for requests, inference (failures included), cache, model loads and batch jobs. 11 alert rules validated by promtool, each on a user-visible symptom. 18-panel Grafana dashboard, auto-provisioned. Prometheus scrapes every API replica and every worker through DNS discovery, verified live with 3 replicas.</t>
         </is>
       </c>
     </row>
@@ -2544,12 +2544,12 @@
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>api/main.py</t>
+          <t>api/</t>
         </is>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>18 documented paths. Verified live through the Docker stack.</t>
+          <t>19 paths in the OpenAPI spec, verified live through the Docker stack.</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>OpenAPI 3.1, 19 paths / 40 schemas. Importable directly into Postman.</t>
+          <t>OpenAPI 3.1, generated from the app, 19 paths. Importable into Postman.</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>95.9% across api/ and worker/ together, the request path end to end: 95.7% on api/, 100% on worker/. 89.3% repo-wide including the training and MLOps code. The async batch endpoint was the last gap at 82.6% and is now fully covered, including the URL fetch with its SSRF checks, the soft-timeout partial-results path and the completion callback at both the helper and its call site.</t>
+          <t>95.8% on api/ and 94.6% on worker/, the whole request and batch path; CI gates api/ at 92%. External services are faked in unit tests (fakeredis, in-memory SQLite, a fake model runtime).</t>
         </is>
       </c>
     </row>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="F58" s="13" t="inlineStr">
         <is>
-          <t>tests/unit/test_image_processing.py</t>
+          <t>tests/unit/test_image_processing.py; tests/unit/test_preprocessing_parity.py</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>27 tests including EXIF orientation, alpha compositing, letterbox round-trip.</t>
+          <t>EXIF orientation, alpha compositing, letterbox round-trip, and training/serving preprocessing parity.</t>
         </is>
       </c>
     </row>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_routes.py</t>
+          <t>tests/unit/test_api_routes.py; tests/unit/test_batch.py</t>
         </is>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>51 tests across every endpoint.</t>
+          <t>Every endpoint, including batch ownership and error envelopes.</t>
         </is>
       </c>
     </row>
@@ -2866,12 +2866,12 @@
       </c>
       <c r="F62" s="13" t="inlineStr">
         <is>
-          <t>tests/integration/test_database.py</t>
+          <t>tests/integration/test_database.py; tests/integration/test_real_services.py</t>
         </is>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>20 tests against real SQL (SQLite).</t>
+          <t>Real SQL against SQLite, and against PostgreSQL and pgvector when reachable (verified).</t>
         </is>
       </c>
     </row>
@@ -2901,12 +2901,12 @@
       </c>
       <c r="F63" s="13" t="inlineStr">
         <is>
-          <t>tests/integration/test_model_loading.py</t>
+          <t>tests/integration/test_model_loading.py; tests/integration/test_quantized_fidelity.py</t>
         </is>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>25 tests against the real ONNX artifacts.</t>
+          <t>Real ONNX artifacts, including every INT8 model against its fp32 twin.</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="F64" s="13" t="inlineStr">
         <is>
-          <t>tests/unit/test_api_routes.py, tests/integration/, scripts/smoke_test_api.py</t>
+          <t>tests/integration/test_api_endpoints.py; tests/e2e/; scripts/smoke_test_api.py</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Plus a verified live run through the Docker stack: 30 checks over every documented endpoint, 30/30 through the gateway and 30/30 against the API's own port. It is a script rather than a transcript, so it reruns against any deployment and exits non-zero on a failure.</t>
+          <t>In-process integration tests plus end-to-end tests through nginx against the running stack, all passing live. smoke_test_api.py checks every endpoint of any deployment and exits non-zero on failure.</t>
         </is>
       </c>
     </row>
@@ -3006,12 +3006,12 @@
       </c>
       <c r="F66" s="13" t="inlineStr">
         <is>
-          <t>tests/performance/test_performance.py</t>
+          <t>tests/performance/test_performance.py; benchmarks/reports/performance_tests.txt</t>
         </is>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>Verified memory levels off over 100 inferences rather than growing linearly.</t>
+          <t>Resident memory measured across repeated inference, batches and preprocessing; growth levels off.</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>366 tests: unit, integration and performance.</t>
+          <t>1,434 tests: 1,230 unit, 161 integration, 28 end-to-end, 15 performance, plus a Locust load test.</t>
         </is>
       </c>
     </row>
@@ -3266,12 +3266,12 @@
       </c>
       <c r="F74" s="13" t="inlineStr">
         <is>
-          <t>.github/workflows/ci.yml</t>
+          <t>.github/workflows/</t>
         </is>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Eight jobs: lint, tests on 3.11 and 3.12, security scan, image build, end-to-end against the deployed stack, real model export. Plus release.yml (publishes attested, scanned images on a version tag) and drift-watch.yml (weekly retraining decision, verified by a manual run).</t>
+          <t>ci.yml: ruff, black and mypy (all enforced), tests on 3.11 and 3.12 with a coverage gate, a strict INT8 fidelity check, security scan, image build and smoke test, end-to-end against the deployed stack, real model export. release.yml publishes scanned, attested images on a tag; drift-watch.yml runs the retraining decision weekly.</t>
         </is>
       </c>
     </row>
@@ -3518,12 +3518,12 @@
       </c>
       <c r="F82" s="13" t="inlineStr">
         <is>
-          <t>docker-compose.yml</t>
+          <t>docker/Dockerfile.worker; worker/</t>
         </is>
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>VERIFIED healthy; processed a real 4-image batch (3 ok, 1 bad image isolated).</t>
+          <t>Healthy in dev and production; batch jobs verified end to end, with job state written to Postgres and metrics served to Prometheus.</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
       </c>
       <c r="G85" s="13" t="inlineStr">
         <is>
-          <t>VERIFIED scraping ml-api; 11 alert rules validated by promtool.</t>
+          <t>Scrapes every API replica and worker; 11 alert rules validated by promtool.</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>VERIFIED: datasource and 22-panel dashboard auto-provisioned.</t>
+          <t>Data source and 18-panel dashboard auto-provisioned.</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>All 7 report healthy. Liveness deliberately checks no dependencies.</t>
+          <t>All 7 dev services and all 10 production containers report healthy, verified live. Liveness checks no dependencies.</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>VERIFIED: all 7 services healthy.</t>
+          <t>All 7 services healthy, verified live.</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>4-step quick start, verified from a clean state.</t>
+          <t>Quick start: clone, git lfs pull, copy .env, docker compose up.</t>
         </is>
       </c>
     </row>
@@ -4151,12 +4151,12 @@
       </c>
       <c r="F101" s="13" t="inlineStr">
         <is>
-          <t>README.md, docs/ASSUMPTIONS.md</t>
+          <t>README.md</t>
         </is>
       </c>
       <c r="G101" s="13" t="inlineStr">
         <is>
-          <t>6 limitations stated plainly; 6 prioritised next steps.</t>
+          <t>7 limitations stated plainly, and next steps in priority order.</t>
         </is>
       </c>
     </row>
@@ -4466,12 +4466,12 @@
       </c>
       <c r="F110" s="13" t="inlineStr">
         <is>
-          <t>docs/ASSUMPTIONS.md</t>
+          <t>docs/ASSUMPTIONS.md; docs/AUDIT.md</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>Brief ambiguities, gaps stated plainly, 3 bugs found in the provided scaffolding and 8 found in my own work.</t>
+          <t>How the brief was read, fixes to 3 provided scripts, and a review against the brief with every issue found and fixed.</t>
         </is>
       </c>
     </row>
@@ -4508,12 +4508,12 @@
       </c>
       <c r="F112" s="13" t="inlineStr">
         <is>
-          <t>pyproject.toml; ruff + black clean</t>
+          <t>pyproject.toml</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>Ruff (13 rule groups) and black pass with zero findings. Every module, class and public function has a docstring explaining WHY, not just what. Each disabled lint rule carries a written reason.</t>
+          <t>ruff, black and mypy all clean and enforced in CI. Each disabled lint rule carries a written reason.</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G113" s="13" t="inlineStr">
         <is>
-          <t>Zero modules below 85% on the critical path, counting worker/ as well as api/: 95.9% across the two, 95.7% on api/, 100% on worker/tasks.py and worker/celery_app.py. 89.3% across the whole repo. The weakest critical-path module is health.py at 86.8%. What remains under 85% is training and MLOps code no request touches: registry.py (a CLI, not imported by api/ or worker/), train_classifier.py, retraining.py, dataset.py, tracking.py.</t>
+          <t>95.8% on api/ and 94.6% on worker/. models/ is 77.2% because it holds the GPU training loop and CLIs that no request touches.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>p99 at batch 1: resnet50 146ms, resnet50-tiny-imagenet 93ms, yolov8n 166ms, embed 63ms. Every model and both precisions stay inside the 1s budget; the slowest overall is yolov8n INT8 at 338ms, 3x inside it.</t>
+          <t>p99 at batch 1: resnet50 211.7 ms, resnet50-tiny-imagenet 277.1 ms, yolov8n 307.5 ms, resnet50-embed 357.3 ms. Every model inside 1 s in both precisions; the slowest single-image p99 is resnet50-embed fp32 at 357.3 ms.</t>
         </is>
       </c>
     </row>
@@ -4648,12 +4648,12 @@
       </c>
       <c r="F116" s="13" t="inlineStr">
         <is>
-          <t>k8s/, docs/TECHNICAL.md, docker-compose.prod.yml</t>
+          <t>k8s/; docs/TECHNICAL.md; docker-compose.prod.yml</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>Stateless API, Redis-backed distributed rate limiting, independent worker scaling, and a pgvector-backed similarity index shared by every replica (the per-process default does not scale, which is why the Kubernetes config sets SIMILARITY_BACKEND=pgvector). Verified on a kind cluster: the HPA scaled ml-api from 1 pod to 2 under a forced target.</t>
+          <t>Stateless API, Redis-backed rate limiting across replicas, independent worker scaling, pgvector similarity index in production and Kubernetes. Production overlay verified live with 3 API replicas and 2 workers; HPA verified on a kind cluster.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor TensorRT quantization and benchmarking in Colab notebook
- Updated the preprocessing configuration to use PREPROCESS_PRESETS for Tiny ImageNet.
- Enhanced the TensorRT engine building process for additional models (ResNet-50, ResNet-50 embedding, YOLOv8n).
- Improved calibration results and updated benchmarks in the documentation.
- Added a new section in the Colab notebook for TensorRT engine building for the additional models.
- Modified the checklist data to reflect the latest performance metrics and model updates.
- Introduced unit tests for benchmarking Torch models against ONNX baselines.
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-26 14:35:36 India Standard Time</t>
+          <t>2026-09-26 15:08:58 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Built and verified on an A100 (TensorRT 11.3.0.99) for the fine-tuned classifier: INT8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms; fp32 1.298 ms. The other three models have CPU INT8 only; building their engines needs another GPU session.</t>
+          <t>Built and verified on an A100 (TensorRT 11.3.0.99) for the fine-tuned classifier: INT8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms; fp32 1.298 ms. The other three models have CPU INT8 only; section 8b of the Colab notebook builds their engines on a GPU runtime and has not been run yet.</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>fp32 and INT8 ONNX for all 4 models at batch 1 and 4, 100 runs per case interleaved across models, plus TensorRT fp32/fp16/INT8. INT8 (uint8, percentile calibration) on this CPU: 1.7x to 2.5x faster than fp32 for the three ResNets, 1.33x slower for yolov8n, 3.67x to 3.92x smaller.</t>
+          <t>Eager PyTorch, ONNX fp32 and ONNX INT8 for all 4 models at batch 1 and 4, 100 runs per case interleaved in one run, plus TensorRT fp32/fp16/INT8. ONNX fp32 is 1.9x to 2.8x faster than PyTorch; INT8 (uint8, percentile) is 2.0x to 2.2x faster again for the ResNets and 1.2x slower for yolov8n, and 3.67x to 3.92x smaller.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>p99 at batch 1: resnet50 211.7 ms, resnet50-tiny-imagenet 277.1 ms, yolov8n 307.5 ms, resnet50-embed 357.3 ms. Every model inside 1 s in both precisions; the slowest single-image p99 is resnet50-embed fp32 at 357.3 ms.</t>
+          <t>p99 at batch 1 in ONNX fp32: resnet50 143.4 ms, resnet50-tiny-imagenet 137.2 ms, yolov8n 186.8 ms, resnet50-embed 84.1 ms. Every model inside 1 s in every runtime; the slowest single-image p99 is eager PyTorch for resnet50-embed at 332.1 ms.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model artifacts and benchmarks for ResNet50 and YOLOv8n
- Enhanced TensorRT model conversion details in checklist_data.py, providing more precise performance metrics for fp32, fp16, and INT8 formats across all models.
- Added new JSON artifact files for ResNet50 and YOLOv8n in fp16, fp32, and INT8 formats, including detailed benchmarking results and agreement metrics with source ONNX models.
- Implemented unit tests to verify the integrity of the engine build process, ensuring that artifacts are correctly fetched and utilized.
- Included additional notes on the precision and performance characteristics of the models, highlighting the differences in behavior across various formats.
</commit_message>
<xml_diff>
--- a/DELIVERABLES_CHECKLIST.xlsx
+++ b/DELIVERABLES_CHECKLIST.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-26 15:08:58 India Standard Time</t>
+          <t>2026-09-26 17:43:31 India Standard Time</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Built and verified on an A100 (TensorRT 11.3.0.99) for the fine-tuned classifier: INT8 0.920 ms p50, 1068 img/s, 24.1 MB; fp16 0.990 ms; fp32 1.298 ms. The other three models have CPU INT8 only; section 8b of the Colab notebook builds their engines on a GPU runtime and has not been run yet.</t>
+          <t>fp32, fp16 and INT8 engines for all 4 models on an A100 (TensorRT 11.3.0.99), batch 1. fp16 is fastest for each (level with INT8 on the fine-tuned classifier): 0.84 to 0.98 ms for the ResNets, 3.16 ms for yolov8n, same answer as fp32 on 98% to 100% of 200 held-out images. INT8 is no faster at batch 1 and agrees with fp32 on 85% to 95% (embeddings: cosine 0.970), close to CPU INT8.</t>
         </is>
       </c>
     </row>

</xml_diff>